<commit_message>
Update split presets and external eval artifacts
</commit_message>
<xml_diff>
--- a/analysis_outputs/rekap_test_external_opensarship1_2_yolov12n_e50_b16.xlsx
+++ b/analysis_outputs/rekap_test_external_opensarship1_2_yolov12n_e50_b16.xlsx
@@ -8,15 +8,17 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test_Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset_Counts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skipped_Rows" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paths" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Per_Class_Evaluation" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset_Counts" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skipped_Rows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paths" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test_Summary'!$A$1:$N$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dataset_Counts'!$A$1:$F$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Skipped_Rows'!$A$1:$D$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Paths'!$A$1:$E$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Per_Class_Evaluation'!$A$1:$I$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Dataset_Counts'!$A$1:$F$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Skipped_Rows'!$A$1:$D$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Paths'!$A$1:$E$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -77,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -88,6 +90,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -672,6 +677,277 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Class_ID</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Class_Name</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Test_Samples</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Precision</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Recall</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>mAP50</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>mAP50-95</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>OpenSARShip-1</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Fishing</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>63</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>0.0044312</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>0.031746</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>0.0077769</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>0.00056955</v>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>0.0001382</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>OpenSARShip-1</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Cargo</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>4120</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>0.88362</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.66165</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>0.75669</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>0.66761</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>0.28232</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>OpenSARShip-1</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Passenger</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>0.0057712</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>0.052632</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>0.010402</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>0.0043984</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>0.0010348</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>OpenSARShip-2</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Fishing</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>204</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>0.003274144469512</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>0.0245098039215686</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>0.0057766187749175</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>0.0008842583463302</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>0.0001763230659178</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>OpenSARShip-2</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Cargo</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>9534</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>0.7844844602079459</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>0.6728550451017411</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>0.7243944529489231</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>0.6274151266505471</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>0.2458120468857941</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>OpenSARShip-2</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Passenger</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>95</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>0.009651508665730901</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>0.09473684210526311</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0.0175183044044603</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>0.0070321189799193</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>0.0020756308113008</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -769,7 +1045,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -872,7 +1148,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>